<commit_message>
test(appium): run and configure mobile e2e test suite with github actions workflow
</commit_message>
<xml_diff>
--- a/reports/appium/TablePulse_Mobile_Appium_Test_Report.xlsx
+++ b/reports/appium/TablePulse_Mobile_Appium_Test_Report.xlsx
@@ -416,7 +416,7 @@
         <v>Project Name</v>
       </c>
       <c r="B2" t="str">
-        <v>TablePulse AI</v>
+        <v>Smart Table AI</v>
       </c>
     </row>
     <row r="3">
@@ -440,7 +440,7 @@
         <v>Execution Date</v>
       </c>
       <c r="B5" t="str">
-        <v>2026-10-05 12:45:30</v>
+        <v>2026-10-13 08:14:45</v>
       </c>
     </row>
     <row r="6">

</xml_diff>